<commit_message>
Ideias antes de Na mídia; quatro destaques de mídia; venda do Buscapé
- Ideias: NeoFeed (IPO e Porsche 930), TechCrunch (fintech, 2017) e o post
  da Headline sobre a Pismo; no inglês, os dois do NeoFeed viram os posts
  equivalentes do Substack
- Ideias vem antes de Na mídia na home e no menu
- Na mídia: quatro destaques (Fortune, Valor, New York Times, Folha);
  midia.py passa a exigir quatro
- Planilha: venda do Buscapé em 2009 pela Exame, Estadão, Folha e IstoÉ
  Dinheiro, mais o perfil da Exame de 2011

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/midia.xlsx
+++ b/data/midia.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veículos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matérias'!$A$1:$P$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Veículos'!$A$1:$E$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matérias'!$A$1:$P$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Veículos'!$A$1:$E$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -168,7 +168,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>1, 2 ou 3 = posição na home. Vazio = fora da home. Precisa haver exatamente três.</t>
+        <t>1 a 4 = posição na home. Vazio = fora da home. Precisa haver exatamente quatro.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -582,6 +582,9 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -596,6 +599,9 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -620,7 +626,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Destaque: 1, 2 e 3 = os três cards da home, nessa ordem. Precisa haver exatamente três.</t>
+          <t>Destaque: 1 a 4 = os quatro cards da home, nessa ordem. Precisa haver exatamente quatro.</t>
         </is>
       </c>
     </row>
@@ -673,10 +679,13 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Uma vez por trimestre: acrescente o que saiu, rode python3 scripts/midia.py check --links e revise os três destaques.</t>
+          <t>Uma vez por trimestre: acrescente o que saiu, rode python3 scripts/midia.py check --links e revise os quatro destaques.</t>
         </is>
       </c>
     </row>
@@ -698,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P92"/>
+  <dimension ref="A1:P97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -809,7 +818,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -848,6 +857,7 @@
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -858,6 +868,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
@@ -908,12 +919,14 @@
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -968,12 +981,14 @@
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1028,8 +1043,10 @@
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1084,8 +1101,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1140,8 +1159,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1196,12 +1217,14 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1256,8 +1279,10 @@
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1312,13 +1337,16 @@
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1363,8 +1391,10 @@
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1419,8 +1449,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1475,8 +1507,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1531,8 +1565,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1587,8 +1623,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1639,8 +1677,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1691,8 +1731,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1743,8 +1785,10 @@
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1795,8 +1839,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1843,8 +1889,10 @@
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1899,8 +1947,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="4" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1955,8 +2005,10 @@
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2007,8 +2059,10 @@
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2063,8 +2117,10 @@
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2119,8 +2175,10 @@
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2175,8 +2233,10 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2231,8 +2291,10 @@
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2287,8 +2349,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2343,8 +2407,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="4" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2399,13 +2465,16 @@
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2450,12 +2519,14 @@
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2510,8 +2581,10 @@
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="4" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2562,8 +2635,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="4" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2618,8 +2693,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="4" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2674,8 +2751,10 @@
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2730,8 +2809,10 @@
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2786,8 +2867,10 @@
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2838,8 +2921,10 @@
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2898,8 +2983,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2958,8 +3045,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3014,8 +3103,10 @@
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" s="5" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
@@ -3066,12 +3157,14 @@
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3126,12 +3219,14 @@
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3182,8 +3277,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3238,12 +3335,14 @@
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3294,12 +3393,14 @@
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3350,8 +3451,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
       <c r="M47" s="4" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3402,8 +3505,10 @@
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" s="4" t="inlineStr"/>
       <c r="M48" s="4" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" s="5" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
@@ -3450,8 +3555,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr"/>
       <c r="M49" s="4" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3506,8 +3613,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" s="4" t="inlineStr"/>
       <c r="M50" s="4" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3558,8 +3667,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" s="4" t="inlineStr"/>
       <c r="M51" s="4" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3614,12 +3725,14 @@
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3674,8 +3787,10 @@
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" s="4" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3726,8 +3841,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr"/>
       <c r="M54" s="4" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3778,8 +3895,10 @@
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" s="4" t="inlineStr"/>
       <c r="M55" s="4" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3830,8 +3949,10 @@
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
       <c r="L56" s="4" t="inlineStr"/>
       <c r="M56" s="4" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3882,8 +4003,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" s="4" t="inlineStr"/>
       <c r="M57" s="4" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3934,8 +4057,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" s="4" t="inlineStr"/>
       <c r="M58" s="4" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
       <c r="O58" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3986,8 +4111,10 @@
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
       <c r="M59" s="4" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
       <c r="O59" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4038,12 +4165,14 @@
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4094,12 +4223,14 @@
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4119,7 +4250,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -4158,6 +4289,7 @@
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -4168,6 +4300,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4218,8 +4351,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
       <c r="L63" s="4" t="inlineStr"/>
       <c r="M63" s="4" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4270,8 +4405,10 @@
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
       <c r="L64" s="4" t="inlineStr"/>
       <c r="M64" s="4" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4322,8 +4459,10 @@
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
       <c r="L65" s="4" t="inlineStr"/>
       <c r="M65" s="4" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
       <c r="O65" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4374,8 +4513,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
       <c r="L66" s="4" t="inlineStr"/>
       <c r="M66" s="4" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
       <c r="O66" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4430,8 +4571,10 @@
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
       <c r="L67" s="4" t="inlineStr"/>
       <c r="M67" s="4" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
       <c r="O67" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4482,12 +4625,14 @@
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
       <c r="O68" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4538,12 +4683,14 @@
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
       <c r="O69" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4563,7 +4710,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -4617,6 +4764,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr"/>
       <c r="O70" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4682,6 +4830,7 @@
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
       <c r="O71" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4739,6 +4888,7 @@
       </c>
       <c r="L72" s="4" t="inlineStr"/>
       <c r="M72" s="4" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
       <c r="O72" s="5" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
@@ -4800,6 +4950,7 @@
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
       <c r="O73" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4857,6 +5008,7 @@
       </c>
       <c r="L74" s="4" t="inlineStr"/>
       <c r="M74" s="4" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4914,6 +5066,7 @@
       </c>
       <c r="L75" s="4" t="inlineStr"/>
       <c r="M75" s="4" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
       <c r="O75" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4971,6 +5124,7 @@
       </c>
       <c r="L76" s="4" t="inlineStr"/>
       <c r="M76" s="4" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
       <c r="O76" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5036,6 +5190,7 @@
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
       <c r="O77" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5097,11 +5252,13 @@
       </c>
       <c r="L78" s="4" t="inlineStr"/>
       <c r="M78" s="4" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
       <c r="O78" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5157,11 +5314,13 @@
         </is>
       </c>
       <c r="M79" s="4" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
       <c r="O79" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr"/>
@@ -5213,6 +5372,7 @@
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
       <c r="O80" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5270,6 +5430,7 @@
       </c>
       <c r="L81" s="4" t="inlineStr"/>
       <c r="M81" s="4" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
       <c r="O81" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5331,11 +5492,13 @@
       </c>
       <c r="L82" s="4" t="inlineStr"/>
       <c r="M82" s="4" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
       <c r="O82" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5387,11 +5550,13 @@
       </c>
       <c r="L83" s="4" t="inlineStr"/>
       <c r="M83" s="4" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
       <c r="O83" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -5447,6 +5612,7 @@
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
       <c r="O84" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5508,11 +5674,13 @@
       </c>
       <c r="L85" s="4" t="inlineStr"/>
       <c r="M85" s="4" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -5568,11 +5736,13 @@
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
       <c r="O86" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -5628,11 +5798,13 @@
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
       <c r="O87" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -5684,11 +5856,13 @@
       </c>
       <c r="L88" s="4" t="inlineStr"/>
       <c r="M88" s="4" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
       <c r="O88" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -5737,8 +5911,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr"/>
       <c r="L89" s="4" t="inlineStr"/>
       <c r="M89" s="4" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
       <c r="O89" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5797,8 +5973,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr"/>
       <c r="L90" s="4" t="inlineStr"/>
       <c r="M90" s="4" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5857,8 +6035,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" s="4" t="inlineStr"/>
       <c r="M91" s="4" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
       <c r="O91" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5917,8 +6097,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" s="4" t="inlineStr"/>
       <c r="M92" s="4" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
       <c r="O92" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5930,8 +6112,310 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr"/>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>2009-10-07</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>IstoÉ Dinheiro</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Uma festa de R$ 600 milhões</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>https://istoedinheiro.com.br/uma-festa-de-r-600-milhoes/</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>movimento</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+      <c r="M93" s="4" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Matéria de capa sobre a venda à Naspers, uma semana depois do fechamento (30/09/2009)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr"/>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>2011-04-03</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Exame</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Mania de grandeza no Buscapé</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>https://exame.com/pme/ele-encontrou-um-grande-negocio/</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+      <c r="M94" s="4" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Entrevista na Exame PME: trajetória, venda à Naspers e relação com os investidores</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>2009-10-04</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Folha de S.Paulo</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Após venda ao Naspers, BuscaPé mira o exterior</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>https://www1.folha.uol.com.br/fsp/dinheiro/fi0410200916.htm</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>movimento</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M95" s="4" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Reportagem de Julio Wiziack, você no centro e com foto. Destaque 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr"/>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>2009-09-30</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Estadão</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Naspers compra o site Buscapé</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>https://www.estadao.com.br/brasil/naspers-compra-o-site-buscape/</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>movimento</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M96" s="4" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Notícia do dia do anúncio, com fala sua</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr"/>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>2009-09-29</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Exame</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Naspers compra BuscaPé por US$ 342 milhões</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>https://exame.com/tecnologia/naspers-compra-buscape-us-342-milhoes-501866/</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>movimento</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+      <c r="M97" s="4" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Notícia do anúncio, com fala sua</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P92"/>
+  <autoFilter ref="A1:P97"/>
   <dataValidations count="9">
     <dataValidation sqref="A2:A2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>
@@ -5945,8 +6429,8 @@
     <dataValidation sqref="M2:M2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use 1, 2 ou 3." type="list">
-      <formula1>"1,2,3"</formula1>
+    <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use um número de 1 a 4." type="list">
+      <formula1>"1,2,3,4"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use perfil, tese, movimento ou portfolio." type="list">
       <formula1>"perfil,tese,movimento,portfolio"</formula1>
@@ -5972,7 +6456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6020,8 +6504,10 @@
           <t>New York Times</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>1</v>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6045,8 +6531,10 @@
           <t>Fortune</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -6070,8 +6558,10 @@
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>3</v>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -6095,8 +6585,10 @@
           <t>TechCrunch</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>4</v>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -6120,8 +6612,10 @@
           <t>NeoFeed</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>5</v>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -6145,8 +6639,10 @@
           <t>Exame</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>6</v>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6170,8 +6666,10 @@
           <t>InfoMoney</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>7</v>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6195,8 +6693,10 @@
           <t>Brazil Journal</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>8</v>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6215,6 +6715,7 @@
           <t>IstoÉ Dinheiro</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
@@ -6233,6 +6734,7 @@
           <t>Projeto Draft</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
@@ -6251,6 +6753,7 @@
           <t>Startups.com.br</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
@@ -6269,6 +6772,7 @@
           <t>Baguete</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
@@ -6287,6 +6791,7 @@
           <t>Tech Monitor</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
@@ -6305,6 +6810,7 @@
           <t>Seu Dinheiro</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
@@ -6323,6 +6829,7 @@
           <t>Startupi</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
@@ -6341,6 +6848,7 @@
           <t>InvestNews</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
@@ -6359,6 +6867,7 @@
           <t>Finsiders</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
@@ -6377,6 +6886,7 @@
           <t>Telesíntese</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
@@ -6395,7 +6905,9 @@
           <t>PrimoCast</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6408,7 +6920,9 @@
           <t>Powercast</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6421,7 +6935,9 @@
           <t>Show Business</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6434,7 +6950,9 @@
           <t>Novo Comércio Cast</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6447,7 +6965,9 @@
           <t>Outliers</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6460,7 +6980,9 @@
           <t>Do Zero ao Topo</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6473,7 +6995,9 @@
           <t>Café com Investidor</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6486,7 +7010,9 @@
           <t>People2Biz</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6499,6 +7025,7 @@
           <t>Endeavor Brasil</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
@@ -6517,7 +7044,9 @@
           <t>Extremos by G4</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6530,7 +7059,9 @@
           <t>Mercado &amp; Opinião</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6543,7 +7074,9 @@
           <t>Ricardo Basaglia</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6556,6 +7089,7 @@
           <t>Cubo Itaú</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" s="4" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
@@ -6574,6 +7108,7 @@
           <t>MMA Global</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
@@ -6592,6 +7127,7 @@
           <t>Redpoint Ventures</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" s="4" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
@@ -6610,6 +7146,7 @@
           <t>Great Hill Partners</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" s="4" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
@@ -6628,6 +7165,7 @@
           <t>Pismo</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
@@ -6640,8 +7178,46 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Folha de S.Paulo</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.folha.uol.com.br</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Estadão</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.estadao.com.br</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E36"/>
+  <autoFilter ref="A1:E38"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use BR ou INT." type="list">
       <formula1>"BR,INT"</formula1>

</xml_diff>

<commit_message>
Na mídia: Folha e Estadão na faixa de veículos da home
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/midia.xlsx
+++ b/data/midia.xlsx
@@ -582,9 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -599,9 +597,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -679,9 +675,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -857,7 +851,6 @@
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -868,7 +861,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
@@ -919,14 +911,12 @@
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -981,14 +971,12 @@
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1043,10 +1031,8 @@
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1101,10 +1087,8 @@
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1159,10 +1143,8 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1217,14 +1199,12 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1279,10 +1259,8 @@
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1337,16 +1315,13 @@
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1391,10 +1366,8 @@
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1449,10 +1422,8 @@
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1507,10 +1478,8 @@
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1565,10 +1534,8 @@
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1623,10 +1590,8 @@
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1677,10 +1642,8 @@
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1731,10 +1694,8 @@
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1785,10 +1746,8 @@
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1839,10 +1798,8 @@
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1889,10 +1846,8 @@
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1947,10 +1902,8 @@
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2005,10 +1958,8 @@
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2059,10 +2010,8 @@
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2117,10 +2066,8 @@
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2175,10 +2122,8 @@
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2233,10 +2178,8 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2291,10 +2234,8 @@
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2349,10 +2290,8 @@
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2407,10 +2346,8 @@
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
       <c r="O29" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2465,16 +2402,13 @@
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2519,14 +2453,12 @@
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2581,10 +2513,8 @@
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="4" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
       <c r="O32" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2635,10 +2565,8 @@
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="4" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2693,10 +2621,8 @@
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
       <c r="O34" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2751,10 +2677,8 @@
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2809,10 +2733,8 @@
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2867,10 +2789,8 @@
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2921,10 +2841,8 @@
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2983,10 +2901,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3045,10 +2961,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3103,10 +3017,8 @@
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" s="5" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
@@ -3157,14 +3069,12 @@
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3219,14 +3129,12 @@
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3277,10 +3185,8 @@
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3335,14 +3241,12 @@
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3393,14 +3297,12 @@
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3451,10 +3353,8 @@
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
       <c r="M47" s="4" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
       <c r="O47" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3505,10 +3405,8 @@
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" s="4" t="inlineStr"/>
       <c r="M48" s="4" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
       <c r="O48" s="5" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
@@ -3555,10 +3453,8 @@
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr"/>
       <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3613,10 +3509,8 @@
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" s="4" t="inlineStr"/>
       <c r="M50" s="4" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3667,10 +3561,8 @@
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" s="4" t="inlineStr"/>
       <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3725,14 +3617,12 @@
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3787,10 +3677,8 @@
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" s="4" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
       <c r="O53" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3841,10 +3729,8 @@
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr"/>
       <c r="M54" s="4" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3895,10 +3781,8 @@
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" s="4" t="inlineStr"/>
       <c r="M55" s="4" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3949,10 +3833,8 @@
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" s="4" t="inlineStr"/>
       <c r="M56" s="4" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4003,10 +3885,8 @@
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" s="4" t="inlineStr"/>
       <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4057,10 +3937,8 @@
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" s="4" t="inlineStr"/>
       <c r="M58" s="4" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4111,10 +3989,8 @@
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
       <c r="M59" s="4" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
       <c r="O59" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4165,14 +4041,12 @@
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4223,14 +4097,12 @@
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
       <c r="O61" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4289,7 +4161,6 @@
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -4300,7 +4171,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
       <c r="O62" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4351,10 +4221,8 @@
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" s="4" t="inlineStr"/>
       <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
       <c r="O63" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4405,10 +4273,8 @@
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" s="4" t="inlineStr"/>
       <c r="M64" s="4" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
       <c r="O64" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4459,10 +4325,8 @@
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
       <c r="L65" s="4" t="inlineStr"/>
       <c r="M65" s="4" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
       <c r="O65" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4513,10 +4377,8 @@
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
       <c r="L66" s="4" t="inlineStr"/>
       <c r="M66" s="4" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
       <c r="O66" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4571,10 +4433,8 @@
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
       <c r="L67" s="4" t="inlineStr"/>
       <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
       <c r="O67" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4625,14 +4485,12 @@
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
       <c r="O68" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4683,14 +4541,12 @@
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
       <c r="O69" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4764,7 +4620,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
       <c r="O70" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4830,7 +4685,6 @@
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
       <c r="O71" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4888,7 +4742,6 @@
       </c>
       <c r="L72" s="4" t="inlineStr"/>
       <c r="M72" s="4" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
       <c r="O72" s="5" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
@@ -4950,7 +4803,6 @@
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
       <c r="O73" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5008,7 +4860,6 @@
       </c>
       <c r="L74" s="4" t="inlineStr"/>
       <c r="M74" s="4" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
       <c r="O74" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5066,7 +4917,6 @@
       </c>
       <c r="L75" s="4" t="inlineStr"/>
       <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
       <c r="O75" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5124,7 +4974,6 @@
       </c>
       <c r="L76" s="4" t="inlineStr"/>
       <c r="M76" s="4" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
       <c r="O76" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5190,7 +5039,6 @@
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
       <c r="O77" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5252,13 +5100,11 @@
       </c>
       <c r="L78" s="4" t="inlineStr"/>
       <c r="M78" s="4" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
       <c r="O78" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5314,13 +5160,11 @@
         </is>
       </c>
       <c r="M79" s="4" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
       <c r="O79" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr"/>
@@ -5372,7 +5216,6 @@
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
       <c r="O80" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5430,7 +5273,6 @@
       </c>
       <c r="L81" s="4" t="inlineStr"/>
       <c r="M81" s="4" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
       <c r="O81" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5492,13 +5334,11 @@
       </c>
       <c r="L82" s="4" t="inlineStr"/>
       <c r="M82" s="4" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
       <c r="O82" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5550,13 +5390,11 @@
       </c>
       <c r="L83" s="4" t="inlineStr"/>
       <c r="M83" s="4" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
       <c r="O83" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -5612,7 +5450,6 @@
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
       <c r="O84" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5674,13 +5511,11 @@
       </c>
       <c r="L85" s="4" t="inlineStr"/>
       <c r="M85" s="4" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -5736,13 +5571,11 @@
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
       <c r="O86" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -5798,13 +5631,11 @@
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
       <c r="O87" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -5856,13 +5687,11 @@
       </c>
       <c r="L88" s="4" t="inlineStr"/>
       <c r="M88" s="4" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
       <c r="O88" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -5911,10 +5740,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" s="4" t="inlineStr"/>
       <c r="M89" s="4" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
       <c r="O89" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5973,10 +5800,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" s="4" t="inlineStr"/>
       <c r="M90" s="4" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6035,10 +5860,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" s="4" t="inlineStr"/>
       <c r="M91" s="4" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
       <c r="O91" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6097,10 +5920,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" s="4" t="inlineStr"/>
       <c r="M92" s="4" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
       <c r="O92" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6155,10 +5976,8 @@
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" s="4" t="inlineStr"/>
       <c r="M93" s="4" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
       <c r="O93" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6213,10 +6032,8 @@
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" s="4" t="inlineStr"/>
       <c r="M94" s="4" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
       <c r="O94" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6275,14 +6092,12 @@
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M95" s="4" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
       <c r="O95" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6337,14 +6152,12 @@
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M96" s="4" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
       <c r="O96" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6399,10 +6212,8 @@
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" s="4" t="inlineStr"/>
       <c r="M97" s="4" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
       <c r="O97" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6504,10 +6315,8 @@
           <t>New York Times</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C2" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6531,10 +6340,8 @@
           <t>Fortune</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C3" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -6558,10 +6365,8 @@
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C4" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -6585,10 +6390,8 @@
           <t>TechCrunch</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C5" s="4" t="n">
+        <v>6</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -6612,10 +6415,8 @@
           <t>NeoFeed</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="C6" s="4" t="n">
+        <v>7</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -6639,10 +6440,8 @@
           <t>Exame</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="C7" s="4" t="n">
+        <v>8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6666,10 +6465,8 @@
           <t>InfoMoney</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="C8" s="4" t="n">
+        <v>9</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6693,10 +6490,8 @@
           <t>Brazil Journal</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="C9" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6715,8 +6510,7 @@
           <t>IstoÉ Dinheiro</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>https://istoedinheiro.com.br</t>
@@ -6734,8 +6528,7 @@
           <t>Projeto Draft</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="n"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>https://www.projetodraft.com</t>
@@ -6753,8 +6546,7 @@
           <t>Startups.com.br</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="n"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>https://startups.com.br</t>
@@ -6772,8 +6564,7 @@
           <t>Baguete</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="n"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>https://www.baguete.com.br</t>
@@ -6791,8 +6582,7 @@
           <t>Tech Monitor</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="n"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>https://www.techmonitor.ai</t>
@@ -6810,8 +6600,7 @@
           <t>Seu Dinheiro</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="n"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>https://www.seudinheiro.com</t>
@@ -6829,8 +6618,7 @@
           <t>Startupi</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="n"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>https://startupi.com.br</t>
@@ -6848,8 +6636,7 @@
           <t>InvestNews</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="n"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>https://investnews.com.br</t>
@@ -6867,8 +6654,7 @@
           <t>Finsiders</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="n"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>https://finsidersbrasil.com.br</t>
@@ -6886,8 +6672,7 @@
           <t>Telesíntese</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="n"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>https://telesintese.com.br</t>
@@ -6905,9 +6690,7 @@
           <t>PrimoCast</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="C20" s="4" t="n"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6920,9 +6703,7 @@
           <t>Powercast</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="C21" s="4" t="n"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6935,9 +6716,7 @@
           <t>Show Business</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="C22" s="4" t="n"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6950,9 +6729,7 @@
           <t>Novo Comércio Cast</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="C23" s="4" t="n"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6965,9 +6742,7 @@
           <t>Outliers</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="C24" s="4" t="n"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6980,9 +6755,7 @@
           <t>Do Zero ao Topo</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="C25" s="4" t="n"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6995,9 +6768,7 @@
           <t>Café com Investidor</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="C26" s="4" t="n"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -7010,9 +6781,7 @@
           <t>People2Biz</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="C27" s="4" t="n"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -7025,8 +6794,7 @@
           <t>Endeavor Brasil</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
+      <c r="C28" s="4" t="n"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>https://endeavor.org.br</t>
@@ -7044,9 +6812,7 @@
           <t>Extremos by G4</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="C29" s="4" t="n"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -7059,9 +6825,7 @@
           <t>Mercado &amp; Opinião</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="C30" s="4" t="n"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -7074,9 +6838,7 @@
           <t>Ricardo Basaglia</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="C31" s="4" t="n"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -7089,8 +6851,7 @@
           <t>Cubo Itaú</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" s="4" t="inlineStr"/>
+      <c r="C32" s="4" t="n"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>https://cubo.network</t>
@@ -7108,8 +6869,7 @@
           <t>MMA Global</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="n"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>https://www.mmaglobal.com</t>
@@ -7127,8 +6887,7 @@
           <t>Redpoint Ventures</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="n"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>https://www.redpoint.com</t>
@@ -7146,8 +6905,7 @@
           <t>Great Hill Partners</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="n"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>https://www.greathillpartners.com</t>
@@ -7165,8 +6923,7 @@
           <t>Pismo</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="n"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>https://www.pismo.io</t>
@@ -7184,8 +6941,14 @@
           <t>Folha de S.Paulo</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Folha de S.Paulo</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>https://www.folha.uol.com.br</t>
@@ -7203,8 +6966,14 @@
           <t>Estadão</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" s="4" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Estadão</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>https://www.estadao.com.br</t>

</xml_diff>

<commit_message>
Na mídia: Estadão (2009 e 2015) e GQ Brasil (2014)
- Estadão: "A trajetória do Buscapé" (Renato Cruz, 30/09/2009) e
  "Após 16 anos, Romero Rodrigues anuncia saída do Buscapé" (18/09/2015)
- GQ Brasil: Empreendedor do Ano no Men of the Year 2014, coluna de
  Nelson Blecher e a lista dos 10 CEOs mais inspiradores; o vídeo do
  prêmio fica só na planilha
- /midia passa de 62 para 67 peças

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/midia.xlsx
+++ b/data/midia.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veículos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matérias'!$A$1:$P$97</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Veículos'!$A$1:$E$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matérias'!$A$1:$P$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Veículos'!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -582,7 +582,9 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -597,7 +599,9 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -675,7 +679,9 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -701,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P97"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -851,6 +857,7 @@
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -861,6 +868,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
@@ -911,12 +919,14 @@
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -971,12 +981,14 @@
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1031,8 +1043,10 @@
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1087,8 +1101,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1143,8 +1159,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1199,12 +1217,14 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1259,8 +1279,10 @@
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1315,13 +1337,16 @@
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1366,8 +1391,10 @@
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1422,8 +1449,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1478,8 +1507,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1534,8 +1565,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1590,8 +1623,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1642,8 +1677,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1694,8 +1731,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1746,8 +1785,10 @@
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1798,8 +1839,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1846,8 +1889,10 @@
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1902,8 +1947,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="4" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -1958,8 +2005,10 @@
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2010,8 +2059,10 @@
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2066,8 +2117,10 @@
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" s="4" t="inlineStr"/>
       <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2122,8 +2175,10 @@
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" s="4" t="inlineStr"/>
       <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2178,8 +2233,10 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2234,8 +2291,10 @@
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
       <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2290,8 +2349,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2346,8 +2407,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="4" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2402,13 +2465,16 @@
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr"/>
       <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2453,12 +2519,14 @@
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2513,8 +2581,10 @@
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr"/>
       <c r="M32" s="4" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2565,8 +2635,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="4" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2621,8 +2693,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr"/>
       <c r="M34" s="4" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2677,8 +2751,10 @@
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2733,8 +2809,10 @@
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr"/>
       <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2789,8 +2867,10 @@
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2841,8 +2921,10 @@
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr"/>
       <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2901,8 +2983,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -2961,8 +3045,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" s="4" t="inlineStr"/>
       <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3017,8 +3103,10 @@
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" s="5" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
@@ -3069,12 +3157,14 @@
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3129,12 +3219,14 @@
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3185,8 +3277,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3241,12 +3335,14 @@
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3297,12 +3393,14 @@
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3353,8 +3451,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
       <c r="M47" s="4" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3405,8 +3505,10 @@
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" s="4" t="inlineStr"/>
       <c r="M48" s="4" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" s="5" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
@@ -3453,8 +3555,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr"/>
       <c r="M49" s="4" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3509,8 +3613,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" s="4" t="inlineStr"/>
       <c r="M50" s="4" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3561,8 +3667,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" s="4" t="inlineStr"/>
       <c r="M51" s="4" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3617,12 +3725,14 @@
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3677,8 +3787,10 @@
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" s="4" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3729,8 +3841,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr"/>
       <c r="M54" s="4" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3781,8 +3895,10 @@
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" s="4" t="inlineStr"/>
       <c r="M55" s="4" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3833,8 +3949,10 @@
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
       <c r="L56" s="4" t="inlineStr"/>
       <c r="M56" s="4" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3885,8 +4003,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" s="4" t="inlineStr"/>
       <c r="M57" s="4" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3937,8 +4057,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" s="4" t="inlineStr"/>
       <c r="M58" s="4" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
       <c r="O58" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -3989,8 +4111,10 @@
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
       <c r="M59" s="4" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
       <c r="O59" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4041,12 +4165,14 @@
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
       <c r="L60" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4097,12 +4223,14 @@
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4161,6 +4289,7 @@
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
       <c r="L62" s="4" t="inlineStr">
         <is>
           <t>x</t>
@@ -4171,6 +4300,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4221,8 +4351,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
       <c r="L63" s="4" t="inlineStr"/>
       <c r="M63" s="4" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4273,8 +4405,10 @@
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
       <c r="L64" s="4" t="inlineStr"/>
       <c r="M64" s="4" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4325,8 +4459,10 @@
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
       <c r="L65" s="4" t="inlineStr"/>
       <c r="M65" s="4" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
       <c r="O65" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4377,8 +4513,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
       <c r="L66" s="4" t="inlineStr"/>
       <c r="M66" s="4" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
       <c r="O66" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4433,8 +4571,10 @@
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
       <c r="L67" s="4" t="inlineStr"/>
       <c r="M67" s="4" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
       <c r="O67" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4485,12 +4625,14 @@
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
       <c r="L68" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
       <c r="O68" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4541,12 +4683,14 @@
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
       <c r="O69" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4620,6 +4764,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr"/>
       <c r="O70" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4685,6 +4830,7 @@
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
       <c r="O71" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4742,6 +4888,7 @@
       </c>
       <c r="L72" s="4" t="inlineStr"/>
       <c r="M72" s="4" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
       <c r="O72" s="5" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
@@ -4803,6 +4950,7 @@
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
       <c r="O73" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4860,6 +5008,7 @@
       </c>
       <c r="L74" s="4" t="inlineStr"/>
       <c r="M74" s="4" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4917,6 +5066,7 @@
       </c>
       <c r="L75" s="4" t="inlineStr"/>
       <c r="M75" s="4" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
       <c r="O75" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -4974,6 +5124,7 @@
       </c>
       <c r="L76" s="4" t="inlineStr"/>
       <c r="M76" s="4" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
       <c r="O76" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5039,6 +5190,7 @@
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
       <c r="O77" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5100,11 +5252,13 @@
       </c>
       <c r="L78" s="4" t="inlineStr"/>
       <c r="M78" s="4" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
       <c r="O78" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5160,11 +5314,13 @@
         </is>
       </c>
       <c r="M79" s="4" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
       <c r="O79" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr"/>
@@ -5216,6 +5372,7 @@
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
       <c r="O80" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5273,6 +5430,7 @@
       </c>
       <c r="L81" s="4" t="inlineStr"/>
       <c r="M81" s="4" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
       <c r="O81" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5334,11 +5492,13 @@
       </c>
       <c r="L82" s="4" t="inlineStr"/>
       <c r="M82" s="4" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
       <c r="O82" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5390,11 +5550,13 @@
       </c>
       <c r="L83" s="4" t="inlineStr"/>
       <c r="M83" s="4" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
       <c r="O83" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -5450,6 +5612,7 @@
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
       <c r="O84" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5511,11 +5674,13 @@
       </c>
       <c r="L85" s="4" t="inlineStr"/>
       <c r="M85" s="4" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -5571,11 +5736,13 @@
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
       <c r="O86" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -5631,11 +5798,13 @@
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
       <c r="O87" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -5687,11 +5856,13 @@
       </c>
       <c r="L88" s="4" t="inlineStr"/>
       <c r="M88" s="4" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
       <c r="O88" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -5740,8 +5911,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr"/>
       <c r="L89" s="4" t="inlineStr"/>
       <c r="M89" s="4" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
       <c r="O89" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5800,8 +5973,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr"/>
       <c r="L90" s="4" t="inlineStr"/>
       <c r="M90" s="4" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5860,8 +6035,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" s="4" t="inlineStr"/>
       <c r="M91" s="4" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
       <c r="O91" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5920,8 +6097,10 @@
           <t>x</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" s="4" t="inlineStr"/>
       <c r="M92" s="4" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
       <c r="O92" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -5976,8 +6155,10 @@
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
       <c r="L93" s="4" t="inlineStr"/>
       <c r="M93" s="4" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
       <c r="O93" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6032,8 +6213,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
       <c r="L94" s="4" t="inlineStr"/>
       <c r="M94" s="4" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
       <c r="O94" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6092,12 +6275,14 @@
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
       <c r="L95" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M95" s="4" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
       <c r="O95" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6152,12 +6337,14 @@
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
       <c r="L96" s="4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
       <c r="M96" s="4" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
       <c r="O96" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6212,8 +6399,10 @@
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
       <c r="L97" s="4" t="inlineStr"/>
       <c r="M97" s="4" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
       <c r="O97" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
@@ -6225,8 +6414,360 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr"/>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>2009-09-30</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Estadão</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>A trajetória do Buscapé</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>https://www.estadao.com.br/link/renato-cruz/a-trajetoria-do-buscape/</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M98" s="4" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Blog Link, por Renato Cruz, no dia da venda: a origem do Buscapé, com falas suas</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr"/>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>2015-09-18</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Estadão</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Após 16 anos, Romero Rodrigues anuncia saída do Buscapé</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>https://www.estadao.com.br/economia/apos-16-anos--romero-rodrigues-anuncia-saida-do-buscape--imp-/</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>movimento</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M99" s="4" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Mesmo fato do Valor de 17/09/2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr"/>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>2014-11-28</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>GQ Brasil</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Romero Rodrigues é o empreendedor do ano no Men of The Year 2014</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>https://gq.globo.com/Men-of-the-Year/noticia/2014/11/romero-rodrigues-e-o-empreendedor-do-ano-no-men-year-2014.html</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" s="4" t="inlineStr"/>
+      <c r="M100" s="4" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Prêmio: Empreendedor do Ano, GQ Men of the Year 2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr"/>
+      <c r="B101" s="4" t="inlineStr"/>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>2014-11-28</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>GQ Brasil</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Romero Rodrigues é o empreendedor do ano no Men of The Year 2014 | MOTY</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>https://gq.globo.com/video/romero-rodrigues-e-o-empreendedor-do-ano-no-men-of-the-year-2014-moty-3789781.ghtml</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr"/>
+      <c r="M101" s="4" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Vídeo do mesmo prêmio. A página traz 05/12/2018, provavelmente data de migração; usei a da matéria. Fica de fora para não repetir o fato</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr"/>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>2014-09-16</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>GQ Brasil</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Ele é o cara</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>https://gq.globo.com/Colunas/Nelson-Blecher/noticia/2014/09/ele-e-o-cara.html</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" s="4" t="inlineStr"/>
+      <c r="M102" s="4" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Coluna de Nelson Blecher: você como símbolo do empreendedor moderno no Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr"/>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>2014-05-03</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>GQ Brasil</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Os 10 CEOs mais inspiradores do Brasil</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>https://gq.globo.com/Prazeres/Poder/noticia/2014/05/os-10-ceos-mais-inspiradores-do-brasil.html</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>perfil</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" s="4" t="inlineStr"/>
+      <c r="M103" s="4" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Ranking da GQ. Você na lista, como CEO global de Comparação de Preços da Naspers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P97"/>
+  <autoFilter ref="A1:P103"/>
   <dataValidations count="9">
     <dataValidation sqref="A2:A2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>
@@ -6267,7 +6808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6315,8 +6856,10 @@
           <t>New York Times</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>1</v>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -6340,8 +6883,10 @@
           <t>Fortune</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -6365,8 +6910,10 @@
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>3</v>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -6390,8 +6937,10 @@
           <t>TechCrunch</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>6</v>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -6415,8 +6964,10 @@
           <t>NeoFeed</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>7</v>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -6440,8 +6991,10 @@
           <t>Exame</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>8</v>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6465,8 +7018,10 @@
           <t>InfoMoney</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>9</v>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6490,8 +7045,10 @@
           <t>Brazil Journal</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>10</v>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6510,7 +7067,8 @@
           <t>IstoÉ Dinheiro</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>https://istoedinheiro.com.br</t>
@@ -6528,7 +7086,8 @@
           <t>Projeto Draft</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>https://www.projetodraft.com</t>
@@ -6546,7 +7105,8 @@
           <t>Startups.com.br</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>https://startups.com.br</t>
@@ -6564,7 +7124,8 @@
           <t>Baguete</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>https://www.baguete.com.br</t>
@@ -6582,7 +7143,8 @@
           <t>Tech Monitor</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>https://www.techmonitor.ai</t>
@@ -6600,7 +7162,8 @@
           <t>Seu Dinheiro</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>https://www.seudinheiro.com</t>
@@ -6618,7 +7181,8 @@
           <t>Startupi</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>https://startupi.com.br</t>
@@ -6636,7 +7200,8 @@
           <t>InvestNews</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>https://investnews.com.br</t>
@@ -6654,7 +7219,8 @@
           <t>Finsiders</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>https://finsidersbrasil.com.br</t>
@@ -6672,7 +7238,8 @@
           <t>Telesíntese</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>https://telesintese.com.br</t>
@@ -6690,7 +7257,9 @@
           <t>PrimoCast</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6703,7 +7272,9 @@
           <t>Powercast</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6716,7 +7287,9 @@
           <t>Show Business</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6729,7 +7302,9 @@
           <t>Novo Comércio Cast</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6742,7 +7317,9 @@
           <t>Outliers</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6755,7 +7332,9 @@
           <t>Do Zero ao Topo</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6768,7 +7347,9 @@
           <t>Café com Investidor</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6781,7 +7362,9 @@
           <t>People2Biz</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6794,7 +7377,8 @@
           <t>Endeavor Brasil</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>https://endeavor.org.br</t>
@@ -6812,7 +7396,9 @@
           <t>Extremos by G4</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6825,7 +7411,9 @@
           <t>Mercado &amp; Opinião</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6838,7 +7426,9 @@
           <t>Ricardo Basaglia</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
           <t>BR</t>
@@ -6851,7 +7441,8 @@
           <t>Cubo Itaú</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>https://cubo.network</t>
@@ -6869,7 +7460,8 @@
           <t>MMA Global</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>https://www.mmaglobal.com</t>
@@ -6887,7 +7479,8 @@
           <t>Redpoint Ventures</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>https://www.redpoint.com</t>
@@ -6905,7 +7498,8 @@
           <t>Great Hill Partners</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>https://www.greathillpartners.com</t>
@@ -6923,7 +7517,8 @@
           <t>Pismo</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>https://www.pismo.io</t>
@@ -6946,8 +7541,10 @@
           <t>Folha de S.Paulo</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n">
-        <v>4</v>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -6971,8 +7568,10 @@
           <t>Estadão</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
-        <v>5</v>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -6985,8 +7584,27 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>GQ Brasil</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://gq.globo.com</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E38"/>
+  <autoFilter ref="A1:E39"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use BR ou INT." type="list">
       <formula1>"BR,INT"</formula1>

</xml_diff>